<commit_message>
Add new Excel files for product names and English-Vietnamese dictionary
- Created 'SICK - ten dong SP can dich.xlsx' to store product names for translation.
- Created 'Tu dien dich EN-VI.xlsx' for English to Vietnamese dictionary entries.
</commit_message>
<xml_diff>
--- a/data/Noi dung SICK/00 CAN SOAT DICH.xlsx
+++ b/data/Noi dung SICK/00 CAN SOAT DICH.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -479,7 +479,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>W12</t>
+          <t>HF transponders</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -494,19 +494,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>W12-2 Laser; W12 Teflon; W12-3; W12; W12-2 AS-i; W12G</t>
+          <t>NXP ICODE SLIX2; Fujitsu MB89R118; Texas Instruments Tag-it HF-I; NXP ICODE SLIX</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>W12-2 Laser; W12 Teflon; W12-3; W12; W12-2 AS-i; W12G</t>
+          <t>NXP ICODE SLIX2; Fujitsu MB89R118; Texas Instruments Tag-it HF-I; NXP ICODE SLIX</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>MLG-2</t>
+          <t>UHF transponders</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -521,12 +521,12 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>RS-485 + 6 x Q + 2 x I/O; 2 x analog + 1 x Q (IO-Link); 3 x Q (IO-Link); RS-485 + 2 x Q (IO-Link); 2 x analog + 2 x Q (IO-Link); 4 x Q (IO-Link)</t>
+          <t>NXP UCODE G2iM; Impinj Monza 4E; NXP UCODE 9xm; Impinj Monza 4QT; Impinj Monza X 8k; NXP UCODE G2XM (+9 tuỳ chọn khác)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>RS-485 + 6 x Q + 2 x I/O; 2 x analog + 1 x Q (IO-Link); 3 x Q (IO-Link); RS-485 + 2 x Q (IO-Link); 2 x analog + 2 x Q (IO-Link); 4 x Q (IO-Link)</t>
+          <t>NXP UCODE G2iM; Impinj Monza 4E; NXP UCODE 9xm; Impinj Monza 4QT; Impinj Monza X 8k; NXP UCODE G2XM (+9 tuỳ chọn khác)</t>
         </is>
       </c>
     </row>
@@ -548,19 +548,19 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>MLGxxNxxxxHxxxxx; MLGxxS-xxxxAx; MLGxxS-xxxxDx; MLGxxN-xxxxNx; MLGxxA-xxxxRx; MLGxxA-xxxxIx (+3 tuỳ chọn khác)</t>
+          <t>2 x analog + 2 x Q (IO-Link); RS-485 + 2 x Q (IO-Link); 4 x Q (IO-Link); RS-485 + 6 x Q + 2 x I/O; 2 x analog + 1 x Q (IO-Link); 3 x Q (IO-Link)</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>MLGxxNxxxxHxxxxx; MLGxxS-xxxxAx; MLGxxS-xxxxDx; MLGxxN-xxxxNx; MLGxxA-xxxxRx; MLGxxA-xxxxIx (+3 tuỳ chọn khác)</t>
+          <t>2 x analog + 2 x Q (IO-Link); RS-485 + 2 x Q (IO-Link); 4 x Q (IO-Link); RS-485 + 6 x Q + 2 x I/O; 2 x analog + 1 x Q (IO-Link); 3 x Q (IO-Link)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>MLG-2 WebChecker</t>
+          <t>MLG-2</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -575,19 +575,19 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>1 x analog + 3 x Q (IO-Link); 2 x analog + 2 x Q (IO-Link); RS-485 + 2 x Q (IO-Link); 4 x Q (IO-Link)</t>
+          <t>MLGxxNxxxxHxxxxx; MLGxxS-xxxxAx; MLGxxN-xxxxEx; MLGxxA-xxxxBx; MLGxxA-xxxxRx; MLGxxA-xxxxIx (+3 tuỳ chọn khác)</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>1 x analog + 3 x Q (IO-Link); 2 x analog + 2 x Q (IO-Link); RS-485 + 2 x Q (IO-Link); 4 x Q (IO-Link)</t>
+          <t>MLGxxNxxxxHxxxxx; MLGxxS-xxxxAx; MLGxxN-xxxxEx; MLGxxA-xxxxBx; MLGxxA-xxxxRx; MLGxxA-xxxxIx (+3 tuỳ chọn khác)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Sensor-actuator cables</t>
+          <t>MLG-2 WebChecker</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -602,24 +602,24 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>M8; D-Sub; M26; RJ45; D-Sub-HD; M12 (+1 tuỳ chọn khác)</t>
+          <t>4 x Q (IO-Link); 1 x analog + 3 x Q (IO-Link); RS-485 + 2 x Q (IO-Link); 2 x analog + 2 x Q (IO-Link)</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>M8; D-Sub; M26; RJ45; D-Sub-HD; M12 (+1 tuỳ chọn khác)</t>
+          <t>4 x Q (IO-Link); 1 x analog + 3 x Q (IO-Link); RS-485 + 2 x Q (IO-Link); 2 x analog + 2 x Q (IO-Link)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Industrial Ethernet cables and fieldbus cables</t>
+          <t>W12</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Mô tả ngắn</t>
+          <t>Giá trị thông số</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -629,24 +629,24 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>PROFIBUS, CANopen, Interbus, PROFINET, EtherNet/IP™ &amp; Gigabit Ethernet</t>
+          <t>W12-3; W12-2 AS-i; W12 Teflon; W12; W12-2 Laser; W12G</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>PROFIBUS, CANopen, Interbus, PROFINET, EtherNet/IP™ &amp; Gigabit Ethernet</t>
+          <t>W12-3; W12-2 AS-i; W12 Teflon; W12; W12-2 Laser; W12G</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>HF transponders</t>
+          <t>Industrial Ethernet cables and fieldbus cables</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Giá trị thông số</t>
+          <t>Mô tả ngắn</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -656,39 +656,12 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Texas Instruments Tag-it HF-I; Fujitsu MB89R118; NXP ICODE SLIX2; NXP ICODE SLIX</t>
+          <t>PROFIBUS, CANopen, Interbus, PROFINET, EtherNet/IP™ &amp; Gigabit Ethernet</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Texas Instruments Tag-it HF-I; Fujitsu MB89R118; NXP ICODE SLIX2; NXP ICODE SLIX</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>HF transponders</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Giá trị thông số</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>chua dich</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Texas Instruments Tag-it HF-I; Fujitsu MB89R118; NXP ICODE SLIX2; NXP ICODE SLIX</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Texas Instruments Tag-it HF-I; Fujitsu MB89R118; NXP ICODE SLIX2; NXP ICODE SLIX</t>
+          <t>PROFIBUS, CANopen, Interbus, PROFINET, EtherNet/IP™ &amp; Gigabit Ethernet</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scripts for translating product names and extracting technical data from PDFs
- Created `sick_name_translate.py` to translate product names from English to Vietnamese, with a focus on maintaining specific product identifiers and translating descriptive terms.
- Implemented functionality to curate existing translations and interact with a language model for generating translations.
- Added `sick_tdo.py` to extract technical data from product overview PDFs, ensuring the correct data is captured from specified sections of the documents.
- Introduced concurrent processing for fetching and parsing PDF data to improve efficiency.
- Added a new Word document `review_sick.docx` for documentation purposes.
</commit_message>
<xml_diff>
--- a/data/Noi dung SICK/00 CAN SOAT DICH.xlsx
+++ b/data/Noi dung SICK/00 CAN SOAT DICH.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -479,7 +479,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>HF transponders</t>
+          <t>FlexChain</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -494,19 +494,19 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>NXP ICODE SLIX2; Fujitsu MB89R118; Texas Instruments Tag-it HF-I; NXP ICODE SLIX</t>
+          <t>IO-Link (V1.1); Serial (RS-485); CANopen; IO-Link; Serial</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>NXP ICODE SLIX2; Fujitsu MB89R118; Texas Instruments Tag-it HF-I; NXP ICODE SLIX</t>
+          <t>IO-Link (V1.1); Serial (RS-485); CANopen; IO-Link; Serial</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>UHF transponders</t>
+          <t>Visionary-B Two</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -521,19 +521,19 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>NXP UCODE G2iM; Impinj Monza 4E; NXP UCODE 9xm; Impinj Monza 4QT; Impinj Monza X 8k; NXP UCODE G2XM (+9 tuỳ chọn khác)</t>
+          <t>SICK AppStudio, SICK AppManager, SOPASair</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>NXP UCODE G2iM; Impinj Monza 4E; NXP UCODE 9xm; Impinj Monza 4QT; Impinj Monza X 8k; NXP UCODE G2XM (+9 tuỳ chọn khác)</t>
+          <t>SICK AppStudio, SICK AppManager, SOPASair</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>MLG-2</t>
+          <t>DFS2x</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -548,24 +548,24 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>2 x analog + 2 x Q (IO-Link); RS-485 + 2 x Q (IO-Link); 4 x Q (IO-Link); RS-485 + 6 x Q + 2 x I/O; 2 x analog + 1 x Q (IO-Link); 3 x Q (IO-Link)</t>
+          <t>TTL / RS-422; HTL / Push pull; Open Collector; TTL / HTL</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>2 x analog + 2 x Q (IO-Link); RS-485 + 2 x Q (IO-Link); 4 x Q (IO-Link); RS-485 + 6 x Q + 2 x I/O; 2 x analog + 1 x Q (IO-Link); 3 x Q (IO-Link)</t>
+          <t>TTL / RS-422; HTL / Push pull; Open Collector; TTL / HTL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>MLG-2</t>
+          <t>Industrial Ethernet cables and fieldbus cables</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Giá trị thông số</t>
+          <t>Mô tả ngắn</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -575,19 +575,19 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>MLGxxNxxxxHxxxxx; MLGxxS-xxxxAx; MLGxxN-xxxxEx; MLGxxA-xxxxBx; MLGxxA-xxxxRx; MLGxxA-xxxxIx (+3 tuỳ chọn khác)</t>
+          <t>PROFIBUS, CANopen, Interbus, PROFINET, EtherNet/IP™ &amp; Gigabit Ethernet</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>MLGxxNxxxxHxxxxx; MLGxxS-xxxxAx; MLGxxN-xxxxEx; MLGxxA-xxxxBx; MLGxxA-xxxxRx; MLGxxA-xxxxIx (+3 tuỳ chọn khác)</t>
+          <t>PROFIBUS, CANopen, Interbus, PROFINET, EtherNet/IP™ &amp; Gigabit Ethernet</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>MLG-2 WebChecker</t>
+          <t>DWS Dynamic</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -602,19 +602,19 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>4 x Q (IO-Link); 1 x analog + 3 x Q (IO-Link); RS-485 + 2 x Q (IO-Link); 2 x analog + 2 x Q (IO-Link)</t>
+          <t>1D; 2D; RFID; PDF417; Aztec; 4-state; Maxi-Code</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>4 x Q (IO-Link); 1 x analog + 3 x Q (IO-Link); RS-485 + 2 x Q (IO-Link); 2 x analog + 2 x Q (IO-Link)</t>
+          <t>1D; 2D; RFID; PDF417; Aztec; 4-state; Maxi-Code</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>W12</t>
+          <t>DWS Pallet</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -629,39 +629,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>W12-3; W12-2 AS-i; W12 Teflon; W12; W12-2 Laser; W12G</t>
+          <t>1D; 2D; PDF417; Aztec; 4-state; Maxi-Code</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>W12-3; W12-2 AS-i; W12 Teflon; W12; W12-2 Laser; W12G</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Industrial Ethernet cables and fieldbus cables</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Mô tả ngắn</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>chua dich</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>PROFIBUS, CANopen, Interbus, PROFINET, EtherNet/IP™ &amp; Gigabit Ethernet</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>PROFIBUS, CANopen, Interbus, PROFINET, EtherNet/IP™ &amp; Gigabit Ethernet</t>
+          <t>1D; 2D; PDF417; Aztec; 4-state; Maxi-Code</t>
         </is>
       </c>
     </row>

</xml_diff>